<commit_message>
implement restoration planning logic
</commit_message>
<xml_diff>
--- a/data/Baseline_cover_EXAMPLE.xlsx
+++ b/data/Baseline_cover_EXAMPLE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\__git\CBuRT\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7B33DA3-E931-4A32-B4B2-0758BFAF6843}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{640D451A-3ED0-4E94-8415-3828602DA506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="1" xr2:uid="{0278FB9D-D97A-43A8-AA68-A0B70EFAF30B}"/>
+    <workbookView xWindow="71895" yWindow="22140" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{0278FB9D-D97A-43A8-AA68-A0B70EFAF30B}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="3" r:id="rId1"/>
@@ -987,7 +987,7 @@
         <v>44</v>
       </c>
       <c r="B2">
-        <v>2.2551546390000001</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="C2" t="s">
         <v>103</v>
@@ -1022,7 +1022,7 @@
         <v>55</v>
       </c>
       <c r="B3">
-        <v>0.19329896899999999</v>
+        <v>0.2</v>
       </c>
       <c r="C3" t="s">
         <v>103</v>
@@ -1057,7 +1057,7 @@
         <v>42</v>
       </c>
       <c r="B4">
-        <v>1.481958763</v>
+        <v>1.5</v>
       </c>
       <c r="C4" t="s">
         <v>103</v>
@@ -1127,7 +1127,7 @@
         <v>58</v>
       </c>
       <c r="B6">
-        <v>0.12886597899999999</v>
+        <v>0.1</v>
       </c>
       <c r="C6" t="s">
         <v>103</v>
@@ -1162,7 +1162,7 @@
         <v>44</v>
       </c>
       <c r="B7">
-        <v>7.7181208049999999</v>
+        <v>7.7</v>
       </c>
       <c r="C7" t="s">
         <v>103</v>
@@ -1677,6 +1677,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="797e7fd4-719a-42b3-b312-968ffa9058ad">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="811eef35-9bdd-441e-81aa-50455f68c6c3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000AA90A7536739341825FB392424435FB" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ca57789ecb406bb7a99068f68ac4c0ed">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="797e7fd4-719a-42b3-b312-968ffa9058ad" xmlns:ns3="811eef35-9bdd-441e-81aa-50455f68c6c3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="89dc4794f4784a0bac47690674a3da53" ns2:_="" ns3:_="">
     <xsd:import namespace="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
@@ -1871,27 +1891,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="797e7fd4-719a-42b3-b312-968ffa9058ad">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="811eef35-9bdd-441e-81aa-50455f68c6c3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D6BB395-747F-41BC-A23A-168993E4FE92}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9D3406C-31AD-4E38-96F6-B0246BC4EAE6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
+    <ds:schemaRef ds:uri="811eef35-9bdd-441e-81aa-50455f68c6c3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D5B4E66-2F53-40AB-B6DF-59838CE46951}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1910,25 +1929,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9D3406C-31AD-4E38-96F6-B0246BC4EAE6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
-    <ds:schemaRef ds:uri="811eef35-9bdd-441e-81aa-50455f68c6c3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D6BB395-747F-41BC-A23A-168993E4FE92}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{6dd02d64-b7f3-43f7-a145-cfd68d338edf}" enabled="1" method="Standard" siteId="{0693b5ba-4b18-4d7b-9341-f32f400a5494}" removed="0"/>

</xml_diff>